<commit_message>
Update: maior peso para o número
Quando encontra um número igual ao procurado dentro das sugestões, dá mais pontos para ele
</commit_message>
<xml_diff>
--- a/source/ago25/rapidfuzz/result_20250902_135716.xlsx
+++ b/source/ago25/rapidfuzz/result_20250902_135716.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Projetos\tcc-culturaeduca\source\ago25\rapidfuzz\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BC59D741-1BEF-48C4-A634-F475FBEE4D18}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{21D369E0-3537-4587-A354-C42DD47984F6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-105" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Enderecos" sheetId="1" r:id="rId1"/>
@@ -23,6 +23,88 @@
 </workbook>
 </file>
 
+<file path=xl/comments1.xml><?xml version="1.0" encoding="utf-8"?>
+<comments xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="xr">
+  <authors>
+    <author>Sabrina Araújo</author>
+  </authors>
+  <commentList>
+    <comment ref="F2" authorId="0" shapeId="0" xr:uid="{89AC32B9-358A-46A1-8B3E-5936662C50C7}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Sabrina Araújo:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Tem na base mas para o bairro CENTRO</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F6" authorId="0" shapeId="0" xr:uid="{3BE0DECC-4142-48DD-A075-2FF0FD15BE80}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Sabrina Araújo:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Na base do CNES tem esse endereço mas com bairro SERRARIA</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="F7" authorId="0" shapeId="0" xr:uid="{4D1D9715-0E96-4D13-A175-15438DC3B17A}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t>Sabrina Araújo:</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="9"/>
+            <color indexed="81"/>
+            <rFont val="Segoe UI"/>
+            <charset val="1"/>
+          </rPr>
+          <t xml:space="preserve">
+Achou na base do Cnes mas para o bairro CONCEICAO</t>
+        </r>
+      </text>
+    </comment>
+  </commentList>
+</comments>
+</file>
+
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="224" uniqueCount="152">
   <si>
@@ -486,7 +568,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="2" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -502,8 +584,21 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="9"/>
+      <color indexed="81"/>
+      <name val="Segoe UI"/>
+      <charset val="1"/>
+    </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -513,6 +608,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="5" tint="0.59999389629810485"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="6" tint="0.59999389629810485"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -544,12 +645,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -853,7 +955,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:M42"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
@@ -906,13 +1008,13 @@
       </c>
     </row>
     <row r="2" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A2" s="2">
+      <c r="A2" s="3">
         <v>30</v>
       </c>
-      <c r="B2" s="2" t="s">
+      <c r="B2" s="3" t="s">
         <v>42</v>
       </c>
-      <c r="C2" s="2">
+      <c r="C2" s="3">
         <v>605</v>
       </c>
       <c r="D2" s="2" t="s">
@@ -959,13 +1061,13 @@
       <c r="D3" s="2" t="s">
         <v>52</v>
       </c>
-      <c r="E3" s="2">
+      <c r="E3" s="3">
         <v>128655</v>
       </c>
-      <c r="F3" s="2" t="s">
+      <c r="F3" s="3" t="s">
         <v>93</v>
       </c>
-      <c r="G3" s="2">
+      <c r="G3" s="3">
         <v>834</v>
       </c>
       <c r="H3" s="2" t="s">
@@ -1000,13 +1102,13 @@
       <c r="D4" s="2" t="s">
         <v>67</v>
       </c>
-      <c r="E4" s="2">
+      <c r="E4" s="3">
         <v>59437</v>
       </c>
-      <c r="F4" s="2" t="s">
+      <c r="F4" s="3" t="s">
         <v>95</v>
       </c>
-      <c r="G4" s="2">
+      <c r="G4" s="3">
         <v>599</v>
       </c>
       <c r="H4" s="2" t="s">
@@ -1041,13 +1143,13 @@
       <c r="D5" s="2" t="s">
         <v>61</v>
       </c>
-      <c r="E5" s="2">
+      <c r="E5" s="3">
         <v>179141</v>
       </c>
-      <c r="F5" s="2" t="s">
+      <c r="F5" s="3" t="s">
         <v>86</v>
       </c>
-      <c r="G5" s="2">
+      <c r="G5" s="3">
         <v>108</v>
       </c>
       <c r="H5" s="2" t="s">
@@ -1070,13 +1172,13 @@
       </c>
     </row>
     <row r="6" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="2">
+      <c r="A6" s="3">
         <v>35</v>
       </c>
-      <c r="B6" s="2" t="s">
+      <c r="B6" s="3" t="s">
         <v>46</v>
       </c>
-      <c r="C6" s="2">
+      <c r="C6" s="3">
         <v>80</v>
       </c>
       <c r="D6" s="2" t="s">
@@ -1111,13 +1213,13 @@
       </c>
     </row>
     <row r="7" spans="1:13" s="2" customFormat="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="2">
+      <c r="A7" s="3">
         <v>21</v>
       </c>
-      <c r="B7" s="2" t="s">
+      <c r="B7" s="3" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="2">
+      <c r="C7" s="3">
         <v>129</v>
       </c>
       <c r="D7" s="2" t="s">
@@ -1164,13 +1266,13 @@
       <c r="D8" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E8" s="2">
+      <c r="E8" s="3">
         <v>43728</v>
       </c>
-      <c r="F8" s="2" t="s">
+      <c r="F8" s="3" t="s">
         <v>101</v>
       </c>
-      <c r="G8" s="2">
+      <c r="G8" s="3">
         <v>763</v>
       </c>
       <c r="H8" s="2" t="s">
@@ -1205,13 +1307,13 @@
       <c r="D9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="E9" s="2">
+      <c r="E9" s="3">
         <v>43091</v>
       </c>
-      <c r="F9" s="2" t="s">
+      <c r="F9" s="3" t="s">
         <v>50</v>
       </c>
-      <c r="G9" s="2">
+      <c r="G9" s="3">
         <v>289</v>
       </c>
       <c r="H9" s="2" t="s">
@@ -1246,13 +1348,13 @@
       <c r="D10" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E10" s="2">
+      <c r="E10" s="3">
         <v>107930</v>
       </c>
-      <c r="F10" s="2" t="s">
+      <c r="F10" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G10" s="2">
+      <c r="G10" s="3">
         <v>615</v>
       </c>
       <c r="H10" s="2" t="s">
@@ -1287,13 +1389,13 @@
       <c r="D11" s="2" t="s">
         <v>51</v>
       </c>
-      <c r="E11" s="2">
+      <c r="E11" s="3">
         <v>107930</v>
       </c>
-      <c r="F11" s="2" t="s">
+      <c r="F11" s="3" t="s">
         <v>72</v>
       </c>
-      <c r="G11" s="2">
+      <c r="G11" s="3">
         <v>615</v>
       </c>
       <c r="H11" s="2" t="s">
@@ -2587,6 +2689,7 @@
     </sortState>
   </autoFilter>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <legacyDrawing r:id="rId1"/>
 </worksheet>
 </file>
 

</xml_diff>